<commit_message>
Add ISB Leadership-with-AI assignment work and academic-assignment-coach skill
- ISB assignments 4.2 (Pinduoduo 5V comparison), 5.2 (servitisation/Maruti),
  6.2 (GenAI in marketing), 10.1 (satellite data/Apollo-Harvesting), 11.2 (Visionary Bank),
  plus 3.2 AT&T roadmap drafts (v2-v6) with instructions, case studies, and versioned drafts
- New skills/aaraminds-academic-assignment-coach skill + README
- Interview Preparations notes; Assignments archive reorganization
</commit_message>
<xml_diff>
--- a/ISB-Leadership-with-AI/Assignments/2_2/Assignment_2_2.xlsx
+++ b/ISB-Leadership-with-AI/Assignments/2_2/Assignment_2_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\aaraminds-education\ISB-Leadership-with-AI\Assignments\2_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CAAFB09-24F3-4068-AE0B-EEA6B7E99DDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E35C85F-7F87-4CA4-8889-7308C12A95DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B7783DF5-699F-4AC1-9907-BF9AC773B06C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Use Case</t>
   </si>
@@ -88,6 +88,13 @@
 Financial &amp; Credit Attributes (Credit limits tied to legal entity, Credit limit expiration dates, Fraud review expiration dates, expected billing dates, Debt/payment-related updates)
 Product &amp; Oppurtunity Context (Product Type, Product categories and configurations)
 Policy &amp; Rule-Based Decision Data (product-specific credit policies, policy thresholds and eligibility rules, policy-driven upates and refresh flows)</t>
+  </si>
+  <si>
+    <t>Consistent Lending Decisions
+Effective default losses with evidence based learning
+Efficient market expansion for thin-file customers
+Quick and fast lending decisions enabling company credibility and better customer satisfaction
+Evidence based analytics for future expansions</t>
   </si>
 </sst>
 </file>
@@ -460,9 +467,29 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{83C085B8-037E-40A9-9D15-948A3CE118CC}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2A1544E-EC6B-4850-9A6E-07D3FCC668D8}">
-  <dimension ref="B2:F38"/>
+  <dimension ref="B2:F37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="41.5703125" customWidth="1"/>
@@ -513,26 +540,28 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="2:6" ht="240" x14ac:dyDescent="0.25">
-      <c r="B6" s="1" t="s">
+    <row r="5" spans="2:6" ht="240" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="F5" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
       <c r="F6" s="1"/>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
@@ -752,13 +781,6 @@
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B38" s="1"/>
-      <c r="C38" s="1"/>
-      <c r="D38" s="1"/>
-      <c r="E38" s="1"/>
-      <c r="F38" s="1"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>